<commit_message>
Fix: force text-format cells per Avito autoload file requirements
</commit_message>
<xml_diff>
--- a/avito-feed/fleet.xlsx
+++ b/avito-feed/fleet.xlsx
@@ -46,8 +46,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -482,341 +483,341 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Уникальный идентификатор объявления</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Начало размещения</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Окончание размещения</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Способ размещения</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Услуга продвижения</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Номер объявления на Авито</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Контактное лицо</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Номер телефона</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Способ связи</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Описание объявления</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Категория</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Цена</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Зоны показа</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Названия фото</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Ссылки на фото</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Ссылка на видео</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Адрес</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Широта</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Долгота</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Название объявления</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Адрес стоянки</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Марка</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Тип кузова</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Модель</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Колёсная формула  [Грузовики]</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Тип двигателя [Грузовики]</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Мощность</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Коробка передач</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Интернет звонки</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Устройства для приёма звонков</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Вид техники</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Валюта</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>НДС включён</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Утильсбор включён</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>Цена в валюте</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Доступность</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>Скидка за лизинг</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>Скидка при покупке от двух единиц</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>Скидка от дилера</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>Доставка</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>Установка дополнительного оборудования</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>Официальная гарантия</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>Дополнительные условия гарантии</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>Подарки</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>URL видеофайла</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>Состояние</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>Пробег</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>ПТС или ПСМ</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>Моточасы</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="AX1" s="1" t="inlineStr">
         <is>
           <t>У шасси и кузова одинаковая марка?</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="AY1" s="1" t="inlineStr">
         <is>
           <t>Тип надстройки</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="AZ1" s="1" t="inlineStr">
         <is>
           <t>Объём кузова</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BA1" s="1" t="inlineStr">
         <is>
           <t>Длина борта</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BB1" s="1" t="inlineStr">
         <is>
           <t>Ширина борта</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="BC1" s="1" t="inlineStr">
         <is>
           <t>Наименование кузовостроителя</t>
         </is>
       </c>
-      <c r="BD1" t="inlineStr">
+      <c r="BD1" s="1" t="inlineStr">
         <is>
           <t>Марка КМУ</t>
         </is>
       </c>
-      <c r="BE1" t="inlineStr">
+      <c r="BE1" s="1" t="inlineStr">
         <is>
           <t>Модель КМУ</t>
         </is>
       </c>
-      <c r="BF1" t="inlineStr">
+      <c r="BF1" s="1" t="inlineStr">
         <is>
           <t>VIN, номер кузова или SN</t>
         </is>
       </c>
-      <c r="BG1" t="inlineStr">
+      <c r="BG1" s="1" t="inlineStr">
         <is>
           <t>Год выпуска</t>
         </is>
       </c>
-      <c r="BH1" t="inlineStr">
+      <c r="BH1" s="1" t="inlineStr">
         <is>
           <t>Грузоподъёмность в кг</t>
         </is>
       </c>
-      <c r="BI1" t="inlineStr">
+      <c r="BI1" s="1" t="inlineStr">
         <is>
           <t>Разрешённая максимальная масса</t>
         </is>
       </c>
-      <c r="BJ1" t="inlineStr">
+      <c r="BJ1" s="1" t="inlineStr">
         <is>
           <t>Объём двигателя</t>
         </is>
       </c>
-      <c r="BK1" t="inlineStr">
+      <c r="BK1" s="1" t="inlineStr">
         <is>
           <t>Экологический класс</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>shacman-sx331863366-px013400</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr"/>
+      <c r="C2" s="1" t="inlineStr"/>
+      <c r="D2" s="1" t="inlineStr"/>
+      <c r="E2" s="1" t="inlineStr"/>
+      <c r="F2" s="1" t="inlineStr"/>
+      <c r="G2" s="1" t="inlineStr"/>
+      <c r="H2" s="1" t="inlineStr"/>
+      <c r="I2" s="1" t="inlineStr">
         <is>
           <t>По телефону и в сообщениях</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="1" t="inlineStr">
         <is>
           <t>Самосвал Shacman SX331863366, 2023 год выпуска.
 Двигатель Weichai WP13.550E501, 550 л.с., дизель.
@@ -827,137 +828,147 @@
 Торг при осмотре.</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="1" t="inlineStr">
         <is>
           <t>Грузовики и спецтехника</t>
         </is>
       </c>
-      <c r="L2" t="n">
-        <v>4500000</v>
-      </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr">
+      <c r="L2" s="1" t="inlineStr">
+        <is>
+          <t>4500000</t>
+        </is>
+      </c>
+      <c r="M2" s="1" t="inlineStr"/>
+      <c r="N2" s="1" t="inlineStr"/>
+      <c r="O2" s="1" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-sx331863366-px013400/side-view.jpeg</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr">
+      <c r="P2" s="1" t="inlineStr"/>
+      <c r="Q2" s="1" t="inlineStr">
         <is>
           <t>Москва, Ижорская ул., 5</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr">
+      <c r="R2" s="1" t="inlineStr"/>
+      <c r="S2" s="1" t="inlineStr"/>
+      <c r="T2" s="1" t="inlineStr"/>
+      <c r="U2" s="1" t="inlineStr"/>
+      <c r="V2" s="1" t="inlineStr">
         <is>
           <t>Shacman</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="W2" s="1" t="inlineStr">
         <is>
           <t>Самосвал</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="X2" s="1" t="inlineStr">
         <is>
           <t>SX331863366</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="Y2" s="1" t="inlineStr">
         <is>
           <t>8×4</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="Z2" s="1" t="inlineStr">
         <is>
           <t>Дизель</t>
         </is>
       </c>
-      <c r="AA2" t="n">
-        <v>550</v>
-      </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AA2" s="1" t="inlineStr">
+        <is>
+          <t>550</t>
+        </is>
+      </c>
+      <c r="AB2" s="1" t="inlineStr">
         <is>
           <t>Механика</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr">
+      <c r="AC2" s="1" t="inlineStr"/>
+      <c r="AD2" s="1" t="inlineStr"/>
+      <c r="AE2" s="1" t="inlineStr">
         <is>
           <t>Грузовики</t>
         </is>
       </c>
-      <c r="AF2" t="inlineStr">
+      <c r="AF2" s="1" t="inlineStr">
         <is>
           <t>RUB</t>
         </is>
       </c>
-      <c r="AG2" t="inlineStr">
+      <c r="AG2" s="1" t="inlineStr">
         <is>
           <t>Нет</t>
         </is>
       </c>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr">
+      <c r="AH2" s="1" t="inlineStr"/>
+      <c r="AI2" s="1" t="inlineStr"/>
+      <c r="AJ2" s="1" t="inlineStr">
         <is>
           <t>В наличии</t>
         </is>
       </c>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="inlineStr"/>
-      <c r="AN2" t="inlineStr"/>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
-      <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr">
+      <c r="AK2" s="1" t="inlineStr"/>
+      <c r="AL2" s="1" t="inlineStr"/>
+      <c r="AM2" s="1" t="inlineStr"/>
+      <c r="AN2" s="1" t="inlineStr"/>
+      <c r="AO2" s="1" t="inlineStr"/>
+      <c r="AP2" s="1" t="inlineStr"/>
+      <c r="AQ2" s="1" t="inlineStr"/>
+      <c r="AR2" s="1" t="inlineStr"/>
+      <c r="AS2" s="1" t="inlineStr"/>
+      <c r="AT2" s="1" t="inlineStr">
         <is>
           <t>С пробегом</t>
         </is>
       </c>
-      <c r="AU2" t="n">
-        <v>123693</v>
-      </c>
-      <c r="AV2" t="inlineStr">
+      <c r="AU2" s="1" t="inlineStr">
+        <is>
+          <t>123693</t>
+        </is>
+      </c>
+      <c r="AV2" s="1" t="inlineStr">
         <is>
           <t>В наличии</t>
         </is>
       </c>
-      <c r="AW2" t="inlineStr"/>
-      <c r="AX2" t="inlineStr">
+      <c r="AW2" s="1" t="inlineStr"/>
+      <c r="AX2" s="1" t="inlineStr">
         <is>
           <t>Да</t>
         </is>
       </c>
-      <c r="AY2" t="inlineStr"/>
-      <c r="AZ2" t="n">
-        <v>35</v>
-      </c>
-      <c r="BA2" t="inlineStr"/>
-      <c r="BB2" t="inlineStr"/>
-      <c r="BC2" t="inlineStr"/>
-      <c r="BD2" t="inlineStr"/>
-      <c r="BE2" t="inlineStr"/>
-      <c r="BF2" t="inlineStr">
+      <c r="AY2" s="1" t="inlineStr"/>
+      <c r="AZ2" s="1" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="BA2" s="1" t="inlineStr"/>
+      <c r="BB2" s="1" t="inlineStr"/>
+      <c r="BC2" s="1" t="inlineStr"/>
+      <c r="BD2" s="1" t="inlineStr"/>
+      <c r="BE2" s="1" t="inlineStr"/>
+      <c r="BF2" s="1" t="inlineStr">
         <is>
           <t>LZGJX4Z61PX013400</t>
         </is>
       </c>
-      <c r="BG2" t="n">
-        <v>2023</v>
-      </c>
-      <c r="BH2" t="inlineStr"/>
-      <c r="BI2" t="inlineStr"/>
-      <c r="BJ2" t="inlineStr"/>
-      <c r="BK2" t="inlineStr">
+      <c r="BG2" s="1" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="BH2" s="1" t="inlineStr"/>
+      <c r="BI2" s="1" t="inlineStr"/>
+      <c r="BJ2" s="1" t="inlineStr"/>
+      <c r="BK2" s="1" t="inlineStr">
         <is>
           <t>Евро 5</t>
         </is>

</xml_diff>

<commit_message>
Add two Shacman X5000 units (93293/97616 km), exclude manually-listed SX331863366
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TkQX9kjSfhXA3jf4gSAGxh
</commit_message>
<xml_diff>
--- a/avito-feed/fleet.xlsx
+++ b/avito-feed/fleet.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BK2"/>
+  <dimension ref="A1:BK3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -440,7 +440,7 @@
     <col width="15" customWidth="1" min="21" max="21"/>
     <col width="10" customWidth="1" min="22" max="22"/>
     <col width="12" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="10" customWidth="1" min="24" max="24"/>
     <col width="31" customWidth="1" min="25" max="25"/>
     <col width="27" customWidth="1" min="26" max="26"/>
     <col width="10" customWidth="1" min="27" max="27"/>
@@ -802,7 +802,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>shacman-sx331863366-px013400</t>
+          <t>shacman-x5000-rx065529</t>
         </is>
       </c>
       <c r="B2" s="1" t="inlineStr"/>
@@ -819,12 +819,16 @@
       </c>
       <c r="J2" s="1" t="inlineStr">
         <is>
-          <t>Самосвал Shacman SX331863366, 2023 год выпуска.
-Двигатель Weichai WP13.550E501, 550 л.с., дизель.
-Колёсная формула 8x4, коробка механическая.
-Пробег 123 693 км, техническое состояние — на ходу, полностью исправен.
-Кузов — самосвал, объём 35 м3.
-Один собственник, эксплуатировался по назначению. Документы в порядке. Смотровая площадка и показ — по договорённости.
+          <t>Самосвал Shacman X5000, 2024 год выпуска.
+Двигатель WP12.550E50, 550 л.с., дизель, объём 11 596 см³, 6 цилиндров, крутящий момент 2060 Н·м, экологический класс Евро 5.
+Колёсная формула 8×4, коробка механическая, 12 передач.
+Пробег 93 293 км, техническое состояние — на ходу, полностью исправен.
+Кузов — самосвал, объём 35 м³ (35000 л).
+Снаряжённая масса 19 500 кг, разрешённая максимальная масса 60 500 кг, грузоподъёмность 41 000 кг.
+Объём топливного бака 500 л, максимальная скорость 80 км/ч.
+Шины 315/80R22.5 (перед/зад).
+Страна происхождения — Китай.
+Документы в порядке. Смотровая площадка и показ — по договорённости.
 Торг при осмотре.</t>
         </is>
       </c>
@@ -835,14 +839,14 @@
       </c>
       <c r="L2" s="1" t="inlineStr">
         <is>
-          <t>4500000</t>
+          <t>7350000</t>
         </is>
       </c>
       <c r="M2" s="1" t="inlineStr"/>
       <c r="N2" s="1" t="inlineStr"/>
       <c r="O2" s="1" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-sx331863366-px013400/side-view.jpeg</t>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065529/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065529/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065529/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065529/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065529/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065529/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065529/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065529/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065529/09.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065529/10.jpg</t>
         </is>
       </c>
       <c r="P2" s="1" t="inlineStr"/>
@@ -867,7 +871,7 @@
       </c>
       <c r="X2" s="1" t="inlineStr">
         <is>
-          <t>SX331863366</t>
+          <t>X5000</t>
         </is>
       </c>
       <c r="Y2" s="1" t="inlineStr">
@@ -930,7 +934,7 @@
       </c>
       <c r="AU2" s="1" t="inlineStr">
         <is>
-          <t>123693</t>
+          <t>93293</t>
         </is>
       </c>
       <c r="AV2" s="1" t="inlineStr">
@@ -957,18 +961,197 @@
       <c r="BE2" s="1" t="inlineStr"/>
       <c r="BF2" s="1" t="inlineStr">
         <is>
-          <t>LZGJX4Z61PX013400</t>
+          <t>LZGJX4Z6XRX065529</t>
         </is>
       </c>
       <c r="BG2" s="1" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="BH2" s="1" t="inlineStr"/>
       <c r="BI2" s="1" t="inlineStr"/>
       <c r="BJ2" s="1" t="inlineStr"/>
       <c r="BK2" s="1" t="inlineStr">
+        <is>
+          <t>Евро 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>shacman-x5000-rx065530</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr"/>
+      <c r="C3" s="1" t="inlineStr"/>
+      <c r="D3" s="1" t="inlineStr"/>
+      <c r="E3" s="1" t="inlineStr"/>
+      <c r="F3" s="1" t="inlineStr"/>
+      <c r="G3" s="1" t="inlineStr"/>
+      <c r="H3" s="1" t="inlineStr"/>
+      <c r="I3" s="1" t="inlineStr">
+        <is>
+          <t>По телефону и в сообщениях</t>
+        </is>
+      </c>
+      <c r="J3" s="1" t="inlineStr">
+        <is>
+          <t>Самосвал Shacman X5000, 2024 год выпуска.
+Двигатель WP12.550E50, 550 л.с., дизель, объём 11 596 см³, 6 цилиндров, крутящий момент 2060 Н·м, экологический класс Евро 5.
+Колёсная формула 8×4, коробка механическая, 12 передач.
+Пробег 97 616 км, техническое состояние — на ходу, полностью исправен.
+Кузов — самосвал, объём 35 м³ (35000 л).
+Снаряжённая масса 19 500 кг, разрешённая максимальная масса 60 500 кг, грузоподъёмность 41 000 кг.
+Объём топливного бака 500 л, максимальная скорость 80 км/ч.
+Шины 315/80R22.5 (перед/зад).
+Страна происхождения — Китай.
+Документы в порядке. Смотровая площадка и показ — по договорённости.
+Торг при осмотре.</t>
+        </is>
+      </c>
+      <c r="K3" s="1" t="inlineStr">
+        <is>
+          <t>Грузовики и спецтехника</t>
+        </is>
+      </c>
+      <c r="L3" s="1" t="inlineStr">
+        <is>
+          <t>7150000</t>
+        </is>
+      </c>
+      <c r="M3" s="1" t="inlineStr"/>
+      <c r="N3" s="1" t="inlineStr"/>
+      <c r="O3" s="1" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065530/01.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065530/02.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065530/03.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065530/04.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065530/05.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065530/06.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065530/07.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065530/08.jpg | https://raw.githubusercontent.com/aj123123-hub/belkar-avito-feed/main/avito-feed/photos/shacman-x5000-rx065530/09.jpg</t>
+        </is>
+      </c>
+      <c r="P3" s="1" t="inlineStr"/>
+      <c r="Q3" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 5</t>
+        </is>
+      </c>
+      <c r="R3" s="1" t="inlineStr"/>
+      <c r="S3" s="1" t="inlineStr"/>
+      <c r="T3" s="1" t="inlineStr"/>
+      <c r="U3" s="1" t="inlineStr"/>
+      <c r="V3" s="1" t="inlineStr">
+        <is>
+          <t>Shacman</t>
+        </is>
+      </c>
+      <c r="W3" s="1" t="inlineStr">
+        <is>
+          <t>Самосвал</t>
+        </is>
+      </c>
+      <c r="X3" s="1" t="inlineStr">
+        <is>
+          <t>X5000</t>
+        </is>
+      </c>
+      <c r="Y3" s="1" t="inlineStr">
+        <is>
+          <t>8×4</t>
+        </is>
+      </c>
+      <c r="Z3" s="1" t="inlineStr">
+        <is>
+          <t>Дизель</t>
+        </is>
+      </c>
+      <c r="AA3" s="1" t="inlineStr">
+        <is>
+          <t>550</t>
+        </is>
+      </c>
+      <c r="AB3" s="1" t="inlineStr">
+        <is>
+          <t>Механика</t>
+        </is>
+      </c>
+      <c r="AC3" s="1" t="inlineStr"/>
+      <c r="AD3" s="1" t="inlineStr"/>
+      <c r="AE3" s="1" t="inlineStr">
+        <is>
+          <t>Грузовики</t>
+        </is>
+      </c>
+      <c r="AF3" s="1" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="AG3" s="1" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="AH3" s="1" t="inlineStr"/>
+      <c r="AI3" s="1" t="inlineStr"/>
+      <c r="AJ3" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AK3" s="1" t="inlineStr"/>
+      <c r="AL3" s="1" t="inlineStr"/>
+      <c r="AM3" s="1" t="inlineStr"/>
+      <c r="AN3" s="1" t="inlineStr"/>
+      <c r="AO3" s="1" t="inlineStr"/>
+      <c r="AP3" s="1" t="inlineStr"/>
+      <c r="AQ3" s="1" t="inlineStr"/>
+      <c r="AR3" s="1" t="inlineStr"/>
+      <c r="AS3" s="1" t="inlineStr"/>
+      <c r="AT3" s="1" t="inlineStr">
+        <is>
+          <t>С пробегом</t>
+        </is>
+      </c>
+      <c r="AU3" s="1" t="inlineStr">
+        <is>
+          <t>97616</t>
+        </is>
+      </c>
+      <c r="AV3" s="1" t="inlineStr">
+        <is>
+          <t>В наличии</t>
+        </is>
+      </c>
+      <c r="AW3" s="1" t="inlineStr"/>
+      <c r="AX3" s="1" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="AY3" s="1" t="inlineStr"/>
+      <c r="AZ3" s="1" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="BA3" s="1" t="inlineStr"/>
+      <c r="BB3" s="1" t="inlineStr"/>
+      <c r="BC3" s="1" t="inlineStr"/>
+      <c r="BD3" s="1" t="inlineStr"/>
+      <c r="BE3" s="1" t="inlineStr"/>
+      <c r="BF3" s="1" t="inlineStr">
+        <is>
+          <t>LZGJX4Z66RX065530</t>
+        </is>
+      </c>
+      <c r="BG3" s="1" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="BH3" s="1" t="inlineStr"/>
+      <c r="BI3" s="1" t="inlineStr"/>
+      <c r="BJ3" s="1" t="inlineStr"/>
+      <c r="BK3" s="1" t="inlineStr">
         <is>
           <t>Евро 5</t>
         </is>

</xml_diff>

<commit_message>
Fix Avito autoload errors: add engine volume, gross weight, currency price
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TkQX9kjSfhXA3jf4gSAGxh
</commit_message>
<xml_diff>
--- a/avito-feed/fleet.xlsx
+++ b/avito-feed/fleet.xlsx
@@ -912,7 +912,11 @@
         </is>
       </c>
       <c r="AH2" s="1" t="inlineStr"/>
-      <c r="AI2" s="1" t="inlineStr"/>
+      <c r="AI2" s="1" t="inlineStr">
+        <is>
+          <t>7350000</t>
+        </is>
+      </c>
       <c r="AJ2" s="1" t="inlineStr">
         <is>
           <t>В наличии</t>
@@ -969,9 +973,21 @@
           <t>2024</t>
         </is>
       </c>
-      <c r="BH2" s="1" t="inlineStr"/>
-      <c r="BI2" s="1" t="inlineStr"/>
-      <c r="BJ2" s="1" t="inlineStr"/>
+      <c r="BH2" s="1" t="inlineStr">
+        <is>
+          <t>41000</t>
+        </is>
+      </c>
+      <c r="BI2" s="1" t="inlineStr">
+        <is>
+          <t>60500</t>
+        </is>
+      </c>
+      <c r="BJ2" s="1" t="inlineStr">
+        <is>
+          <t>11596</t>
+        </is>
+      </c>
       <c r="BK2" s="1" t="inlineStr">
         <is>
           <t>Евро 5</t>
@@ -1091,7 +1107,11 @@
         </is>
       </c>
       <c r="AH3" s="1" t="inlineStr"/>
-      <c r="AI3" s="1" t="inlineStr"/>
+      <c r="AI3" s="1" t="inlineStr">
+        <is>
+          <t>7150000</t>
+        </is>
+      </c>
       <c r="AJ3" s="1" t="inlineStr">
         <is>
           <t>В наличии</t>
@@ -1148,9 +1168,21 @@
           <t>2024</t>
         </is>
       </c>
-      <c r="BH3" s="1" t="inlineStr"/>
-      <c r="BI3" s="1" t="inlineStr"/>
-      <c r="BJ3" s="1" t="inlineStr"/>
+      <c r="BH3" s="1" t="inlineStr">
+        <is>
+          <t>41000</t>
+        </is>
+      </c>
+      <c r="BI3" s="1" t="inlineStr">
+        <is>
+          <t>60500</t>
+        </is>
+      </c>
+      <c r="BJ3" s="1" t="inlineStr">
+        <is>
+          <t>11596</t>
+        </is>
+      </c>
       <c r="BK3" s="1" t="inlineStr">
         <is>
           <t>Евро 5</t>

</xml_diff>

<commit_message>
Fix address to match confirmed Avito business address (Ижорская ул., 15с2)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TkQX9kjSfhXA3jf4gSAGxh
</commit_message>
<xml_diff>
--- a/avito-feed/fleet.xlsx
+++ b/avito-feed/fleet.xlsx
@@ -433,7 +433,7 @@
     <col width="15" customWidth="1" min="14" max="14"/>
     <col width="40" customWidth="1" min="15" max="15"/>
     <col width="17" customWidth="1" min="16" max="16"/>
-    <col width="25" customWidth="1" min="17" max="17"/>
+    <col width="28" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="10" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
@@ -852,7 +852,7 @@
       <c r="P2" s="1" t="inlineStr"/>
       <c r="Q2" s="1" t="inlineStr">
         <is>
-          <t>Москва, Ижорская ул., 5</t>
+          <t>Москва, Ижорская ул., 15с2</t>
         </is>
       </c>
       <c r="R2" s="1" t="inlineStr"/>
@@ -1047,7 +1047,7 @@
       <c r="P3" s="1" t="inlineStr"/>
       <c r="Q3" s="1" t="inlineStr">
         <is>
-          <t>Москва, Ижорская ул., 5</t>
+          <t>Москва, Ижорская ул., 15с2</t>
         </is>
       </c>
       <c r="R3" s="1" t="inlineStr"/>

</xml_diff>

<commit_message>
Add "no repairs needed" line to both descriptions
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TkQX9kjSfhXA3jf4gSAGxh
</commit_message>
<xml_diff>
--- a/avito-feed/fleet.xlsx
+++ b/avito-feed/fleet.xlsx
@@ -822,7 +822,7 @@
           <t>Самосвал Shacman X5000, 2024 год выпуска.
 Двигатель WP12.550E50, 550 л.с., дизель, объём 11 596 см³, 6 цилиндров, крутящий момент 2060 Н·м, экологический класс Евро 5.
 Колёсная формула 8×4, коробка механическая, 12 передач.
-Пробег 93 293 км, техническое состояние — на ходу, полностью исправен.
+Пробег 93 293 км, техническое состояние — на ходу, полностью исправен, не требует вложений и ремонта.
 Кузов — самосвал, объём 35 м³ (35000 л).
 Снаряжённая масса 19 500 кг, разрешённая максимальная масса 60 500 кг, грузоподъёмность 41 000 кг.
 Объём топливного бака 500 л, максимальная скорость 80 км/ч.
@@ -1017,7 +1017,7 @@
           <t>Самосвал Shacman X5000, 2024 год выпуска.
 Двигатель WP12.550E50, 550 л.с., дизель, объём 11 596 см³, 6 цилиндров, крутящий момент 2060 Н·м, экологический класс Евро 5.
 Колёсная формула 8×4, коробка механическая, 12 передач.
-Пробег 97 616 км, техническое состояние — на ходу, полностью исправен.
+Пробег 97 616 км, техническое состояние — на ходу, полностью исправен, не требует вложений и ремонта.
 Кузов — самосвал, объём 35 м³ (35000 л).
 Снаряжённая масса 19 500 кг, разрешённая максимальная масса 60 500 кг, грузоподъёмность 41 000 кг.
 Объём топливного бака 500 л, максимальная скорость 80 км/ч.

</xml_diff>

<commit_message>
Reprice Shacman X5000 trucks to match current used-market comps; save comp table to pricing/
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KRzo6JwTr8ExLnQ6Y4iSPg
</commit_message>
<xml_diff>
--- a/avito-feed/fleet.xlsx
+++ b/avito-feed/fleet.xlsx
@@ -839,7 +839,7 @@
       </c>
       <c r="L2" s="1" t="inlineStr">
         <is>
-          <t>7350000</t>
+          <t>6200000</t>
         </is>
       </c>
       <c r="M2" s="1" t="inlineStr"/>
@@ -914,7 +914,7 @@
       <c r="AH2" s="1" t="inlineStr"/>
       <c r="AI2" s="1" t="inlineStr">
         <is>
-          <t>7350000</t>
+          <t>6200000</t>
         </is>
       </c>
       <c r="AJ2" s="1" t="inlineStr">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="L3" s="1" t="inlineStr">
         <is>
-          <t>7150000</t>
+          <t>5950000</t>
         </is>
       </c>
       <c r="M3" s="1" t="inlineStr"/>
@@ -1109,7 +1109,7 @@
       <c r="AH3" s="1" t="inlineStr"/>
       <c r="AI3" s="1" t="inlineStr">
         <is>
-          <t>7150000</t>
+          <t>5950000</t>
         </is>
       </c>
       <c r="AJ3" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Lower Shacman X5000 prices again after zero contacts in 3 days
</commit_message>
<xml_diff>
--- a/avito-feed/fleet.xlsx
+++ b/avito-feed/fleet.xlsx
@@ -839,7 +839,7 @@
       </c>
       <c r="L2" s="1" t="inlineStr">
         <is>
-          <t>6200000</t>
+          <t>5890000</t>
         </is>
       </c>
       <c r="M2" s="1" t="inlineStr"/>
@@ -914,7 +914,7 @@
       <c r="AH2" s="1" t="inlineStr"/>
       <c r="AI2" s="1" t="inlineStr">
         <is>
-          <t>6200000</t>
+          <t>5890000</t>
         </is>
       </c>
       <c r="AJ2" s="1" t="inlineStr">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="L3" s="1" t="inlineStr">
         <is>
-          <t>5950000</t>
+          <t>5690000</t>
         </is>
       </c>
       <c r="M3" s="1" t="inlineStr"/>
@@ -1109,7 +1109,7 @@
       <c r="AH3" s="1" t="inlineStr"/>
       <c r="AI3" s="1" t="inlineStr">
         <is>
-          <t>5950000</t>
+          <t>5690000</t>
         </is>
       </c>
       <c r="AJ3" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Add missing "Адрес стоянки" to truck feed
Same required field we discovered missing on the trailer feed earlier
today. Both Shacman trucks are currently showing status "old" — this
field was likely part of why the scheduled reprocess didn't keep them
active, given the exact same error already hit trailers today.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WGw8UdFgVU8PXaQaPUvEwH
</commit_message>
<xml_diff>
--- a/avito-feed/fleet.xlsx
+++ b/avito-feed/fleet.xlsx
@@ -437,7 +437,7 @@
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="10" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
-    <col width="15" customWidth="1" min="21" max="21"/>
+    <col width="28" customWidth="1" min="21" max="21"/>
     <col width="10" customWidth="1" min="22" max="22"/>
     <col width="12" customWidth="1" min="23" max="23"/>
     <col width="10" customWidth="1" min="24" max="24"/>
@@ -858,7 +858,11 @@
       <c r="R2" s="1" t="inlineStr"/>
       <c r="S2" s="1" t="inlineStr"/>
       <c r="T2" s="1" t="inlineStr"/>
-      <c r="U2" s="1" t="inlineStr"/>
+      <c r="U2" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
       <c r="V2" s="1" t="inlineStr">
         <is>
           <t>Shacman</t>
@@ -1053,7 +1057,11 @@
       <c r="R3" s="1" t="inlineStr"/>
       <c r="S3" s="1" t="inlineStr"/>
       <c r="T3" s="1" t="inlineStr"/>
-      <c r="U3" s="1" t="inlineStr"/>
+      <c r="U3" s="1" t="inlineStr">
+        <is>
+          <t>Москва, Ижорская ул., 15с2</t>
+        </is>
+      </c>
       <c r="V3" s="1" t="inlineStr">
         <is>
           <t>Shacman</t>

</xml_diff>